<commit_message>
test(1d): fixture anggaran realistis (unik akun-bulan), uji pelari
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/services/integrator/internal/document/testdata/anggaran-dagang-2026-06-batas-hari.golden.xlsx
+++ b/services/integrator/internal/document/testdata/anggaran-dagang-2026-06-batas-hari.golden.xlsx
@@ -227,13 +227,13 @@
         <v>10</v>
       </c>
       <c r="B7" s="7">
-        <v>6500000.33</v>
+        <v>3000000</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
       </c>
       <c r="D7" s="7">
-        <v>-6500000.33</v>
+        <v>-3000000</v>
       </c>
       <c r="E7" s="8">
         <v>-100</v>
@@ -247,13 +247,13 @@
         <v>12</v>
       </c>
       <c r="B8" s="10">
-        <v>6500000.33</v>
+        <v>3000000</v>
       </c>
       <c r="C8" s="10">
         <v>0</v>
       </c>
       <c r="D8" s="10">
-        <v>-6500000.33</v>
+        <v>-3000000</v>
       </c>
       <c r="E8" s="11">
         <v>-100</v>

</xml_diff>